<commit_message>
add bilingual EN/ES toggle to portfolio
</commit_message>
<xml_diff>
--- a/Pulse research exercise/pulse_research_news_tracker.xlsx
+++ b/Pulse research exercise/pulse_research_news_tracker.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -747,6 +747,116 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Molly White launches Tech Influence Watch to track AI spending in politics</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Citationneeded.news</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.citationneeded.news/tech-influence-watch/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Martin Scorsese Slammed by Art Directors Guild for AI Support: ‘A Betrayal of the Collaborative Nature of Cinema’</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TheWrap</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.thewrap.com/creative-content/movies/martin-scorsese-slammed-art-directors-guild-ai-support/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Kedaara Capital slows investments, tightens underwriting amid valuation mismatch</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Livemint</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.livemint.com/companies/kedaara-capital-slows-dealmaking-as-private-market-valuations-stay-high-11780817896294.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>India can take the lead in applying AI in industries: SAP CEO Christian Klein</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>The Times of India</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/tech/artificial-intelligence/india-can-take-the-lead-in-applying-ai-in-industries-sap-ceo-christian-klein/articleshow/131619502.cms</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>AI agents to match physical workforce at TCS soon: Chairman N Chandrasekaran</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The Indian Express</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://indianexpress.com/article/business/companies/ai-agents-to-match-physical-workforce-at-tcs-soon-chairman-n-chandrasekaran-10732210/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>